<commit_message>
updated app with better data checks. Improved Emission calculations to avoid inefficient rowwise()
</commit_message>
<xml_diff>
--- a/inst/extdata/mocaredd-templatev2-simple.xlsx
+++ b/inst/extdata/mocaredd-templatev2-simple.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gaelsola/code/mocaredd.dev2/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF69B15E-BA70-D942-869D-8261BA7874B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2858CE-A328-7E47-B562-DCC7E33416EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="660" windowWidth="28200" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="660" windowWidth="28200" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="11" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="63">
   <si>
     <t>trunc_pdf</t>
   </si>
@@ -442,6 +442,12 @@
   <si>
     <t>digits</t>
   </si>
+  <si>
+    <t>ratio</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
 </sst>
 </file>
 
@@ -606,7 +612,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -644,6 +650,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -928,90 +937,83 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:H1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="21" width="10.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="20" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="20" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2">
         <v>10000</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="b">
+      <c r="D2" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="F2" s="2">
+      <c r="E2" s="2">
         <v>0.9</v>
       </c>
-      <c r="G2">
+      <c r="F2">
         <v>3</v>
       </c>
-      <c r="H2" s="1">
+      <c r="G2" s="1">
         <v>1</v>
       </c>
-      <c r="I2" s="2" t="b">
+      <c r="H2" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="4" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="5" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="6" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="7" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="8" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="9" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="10" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="11" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="12" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="13" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="14" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="15" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="16" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="3" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="4" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="6" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="7" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="8" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="9" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="10" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="12" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="13" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="14" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="15" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="16" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="17" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="18" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="19" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -4457,20 +4459,21 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.5" customWidth="1"/>
-    <col min="8" max="10" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" customWidth="1"/>
+    <col min="7" max="7" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5" customWidth="1"/>
+    <col min="9" max="11" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>33</v>
       </c>
@@ -4478,31 +4481,34 @@
         <v>34</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="E1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -4510,25 +4516,28 @@
         <v>10</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="7">
+      <c r="E2" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="7">
         <v>274.959</v>
       </c>
-      <c r="F2" s="7">
+      <c r="G2" s="7">
         <v>71.765000000000001</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="7"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -4536,25 +4545,28 @@
         <v>10</v>
       </c>
       <c r="C3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="7">
+      <c r="E3" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="7">
         <v>195.58000000000004</v>
       </c>
-      <c r="F3" s="7">
+      <c r="G3" s="7">
         <v>48.006000000000007</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -4562,25 +4574,28 @@
         <v>10</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="8">
+      <c r="E4" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="8">
         <v>0.33300000000000002</v>
       </c>
-      <c r="F4" s="8">
+      <c r="G4" s="8">
         <v>3.0800000000000004E-2</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="H4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="8"/>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -4588,25 +4603,28 @@
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="8">
+      <c r="E5" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="8">
         <v>0.40700000000000003</v>
       </c>
-      <c r="F5" s="8">
+      <c r="G5" s="8">
         <v>3.0800000000000004E-2</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -4614,31 +4632,34 @@
         <v>10</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="E6" s="7">
+      <c r="E6" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" s="7">
         <v>0.72</v>
       </c>
-      <c r="F6" s="7">
+      <c r="G6" s="7">
         <v>0.16200000000000001</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H6" s="7">
-        <f t="shared" ref="H6:H7" si="0">ROUND((E6*(1-E6)/(F6*F6)-1)*E6,3)</f>
+      <c r="I6" s="7">
+        <f t="shared" ref="I6:I7" si="0">ROUND((F6*(1-F6)/(G6*G6)-1)*F6,3)</f>
         <v>4.8109999999999999</v>
       </c>
-      <c r="I6" s="7">
-        <f t="shared" ref="I6:I7" si="1">ROUND((E6*(1-E6)/(F6*F6)-1)*(1-E6),3)</f>
+      <c r="J6" s="7">
+        <f t="shared" ref="J6:J7" si="1">ROUND((F6*(1-F6)/(G6*G6)-1)*(1-F6),3)</f>
         <v>1.871</v>
       </c>
-      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A7" s="7">
         <v>6</v>
       </c>
@@ -4646,31 +4667,34 @@
         <v>10</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="7">
+      <c r="E7" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" s="7">
         <v>0.72</v>
       </c>
-      <c r="F7" s="7">
+      <c r="G7" s="7">
         <v>0.20699999999999999</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="7">
+      <c r="I7" s="7">
         <f t="shared" si="0"/>
         <v>2.6680000000000001</v>
       </c>
-      <c r="I7" s="7">
+      <c r="J7" s="7">
         <f t="shared" si="1"/>
         <v>1.0369999999999999</v>
       </c>
-      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A8" s="7">
         <v>7</v>
       </c>
@@ -4678,25 +4702,28 @@
         <v>10</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="9">
-        <v>0</v>
+      <c r="E8" s="25" t="s">
+        <v>62</v>
       </c>
       <c r="F8" s="9">
         <v>0</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="9">
+        <v>0</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="9"/>
       <c r="I8" s="9"/>
-      <c r="J8" s="10"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="10"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A9" s="7">
         <v>8</v>
       </c>
@@ -4704,18 +4731,21 @@
         <v>10</v>
       </c>
       <c r="C9" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="1">
+      <c r="E9" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="1">
         <v>0.47</v>
       </c>
-      <c r="F9" s="1">
+      <c r="G9" s="1">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>